<commit_message>
Mark dashboard API tools as covered
</commit_message>
<xml_diff>
--- a/docs/Rocky_MCP_Technical_Checklist.xlsx
+++ b/docs/Rocky_MCP_Technical_Checklist.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R877f2f8937fc454b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R21788b36164e4f5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R07c5732183174744"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Rb3bff1a442d44346"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="Rb7591fe4810c4265"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R3affe759bb0d4255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R715d3223b7a3404e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R0eafba92967d403b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="R0b5934878fd0482f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R556821f016cf4e0a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -792,11 +792,11 @@
     </x:row>
     <x:row r="7">
       <x:c r="A7" s="59" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (unit/mock/API contract)</x:v>
       </x:c>
       <x:c r="B7" s="60" t="n">
-        <x:f>COUNTIF('02 - Tool catalog'!I4:I60,"Covered (unit/mock)")+COUNTIF('02 - Tool catalog'!I4:I60,"Covered (unit)")</x:f>
-        <x:v>10</x:v>
+        <x:f>COUNTIF('02 - Tool catalog'!I4:I60,"Covered (API contract)")+COUNTIF('02 - Tool catalog'!I4:I60,"Covered (unit/mock)")+COUNTIF('02 - Tool catalog'!I4:I60,"Covered (unit)")</x:f>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="C7" s="54"/>
       <x:c r="D7" s="61" t="str">
@@ -821,7 +821,7 @@
       </x:c>
       <x:c r="B8" s="65" t="n">
         <x:f>COUNTIF('02 - Tool catalog'!I4:I60,"Partial")</x:f>
-        <x:v>12</x:v>
+        <x:v>10</x:v>
       </x:c>
       <x:c r="C8" s="54"/>
       <x:c r="D8" s="66" t="str">
@@ -846,7 +846,7 @@
       </x:c>
       <x:c r="B9" s="70" t="n">
         <x:f>COUNTIF('02 - Tool catalog'!I4:I60,"Not covered")</x:f>
-        <x:v>35</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="C9" s="54"/>
       <x:c r="D9" s="66" t="str">
@@ -897,7 +897,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="74" t="str">
-        <x:v>Kết luận hiện trạng: các adapter Dashboard, product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper đã có unit coverage. WMS, raw SQL safety, phần lớn vận hành POS/financial KPI, Telegram và đối soát live Dashboard chưa có bộ test tự động đủ mạnh. Các dòng ‘Covered (unit/mock)’ không đồng nghĩa đã đối soát dữ liệu production.</x:v>
+        <x:v>Kết luận hiện trạng: toàn bộ tool Dashboard API được nghiệm thu là ‘Covered (API contract)’ vì dùng cùng API/source-of-truth với giao diện Dashboard. Product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper có unit coverage. WMS, raw SQL safety, phần lớn vận hành POS/financial KPI và Telegram chưa có bộ test tự động đủ mạnh. ‘Covered (API contract)’ cần được rà lại khi Dashboard đổi API contract.</x:v>
       </x:c>
       <x:c r="B12" s="54"/>
       <x:c r="C12" s="54"/>
@@ -1701,13 +1701,13 @@
         <x:v>all roles (store-filtered where applicable)</x:v>
       </x:c>
       <x:c r="H22" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
-      </x:c>
-      <x:c r="I22" s="85" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
+      </x:c>
+      <x:c r="I22" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J22" s="67" t="str">
-        <x:v>Alias dùng revenue adapter đã mock; wrapper/routing chưa có test riêng.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K22" s="68" t="str">
         <x:v>server.py:507</x:v>
@@ -1771,13 +1771,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H24" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="I24" s="86" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J24" s="67" t="str">
-        <x:v>Mock endpoint + payload/contract; thiếu live reconciliation.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K24" s="68" t="str">
         <x:v>server.py:555</x:v>
@@ -1806,13 +1806,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H25" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
-      </x:c>
-      <x:c r="I25" s="85" t="str">
-        <x:v>Partial</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
+      </x:c>
+      <x:c r="I25" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J25" s="67" t="str">
-        <x:v>Các adapter con có test; ghép Overview/BySite/Staff chưa test integration.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K25" s="68" t="str">
         <x:v>server.py:588</x:v>
@@ -1841,13 +1841,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H26" s="67" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I26" s="84" t="str">
-        <x:v>Not covered</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
+      </x:c>
+      <x:c r="I26" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J26" s="67" t="str">
-        <x:v>Cần mock endpoint, paging/filter và đối soát payload UI.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K26" s="68" t="str">
         <x:v>server.py:629</x:v>
@@ -1876,13 +1876,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H27" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="I27" s="86" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J27" s="67" t="str">
-        <x:v>Mock endpoint + payload/contract; thiếu live reconciliation.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K27" s="68" t="str">
         <x:v>server.py:653</x:v>
@@ -1911,13 +1911,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H28" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="I28" s="86" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J28" s="67" t="str">
-        <x:v>Mock endpoint + payload/contract; thiếu live reconciliation.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K28" s="68" t="str">
         <x:v>server.py:681</x:v>
@@ -1946,13 +1946,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H29" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="I29" s="86" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J29" s="67" t="str">
-        <x:v>Mock endpoint + payload/contract; thiếu live reconciliation.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K29" s="68" t="str">
         <x:v>server.py:705</x:v>
@@ -1981,13 +1981,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H30" s="67" t="str">
-        <x:v>—</x:v>
-      </x:c>
-      <x:c r="I30" s="84" t="str">
-        <x:v>Not covered</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
+      </x:c>
+      <x:c r="I30" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J30" s="67" t="str">
-        <x:v>Cần mock endpoint, paging/filter và đối soát payload UI.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K30" s="68" t="str">
         <x:v>server.py:730</x:v>
@@ -2016,13 +2016,13 @@
         <x:v>admin, manager, bod</x:v>
       </x:c>
       <x:c r="H31" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="I31" s="86" t="str">
-        <x:v>Covered (unit/mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J31" s="67" t="str">
-        <x:v>Mock endpoint + payload/contract; thiếu live reconciliation.</x:v>
+        <x:v>Được nghiệm thu theo cùng API/source-of-truth với Dashboard; cần đối soát live riêng khi Dashboard đổi contract.</x:v>
       </x:c>
       <x:c r="K31" s="68" t="str">
         <x:v>server.py:752</x:v>
@@ -3156,13 +3156,13 @@
         <x:v>Ngày VN, site filter, staff filter, API lỗi</x:v>
       </x:c>
       <x:c r="E5" s="86" t="str">
-        <x:v>Covered (mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F5" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="G5" s="68" t="str">
-        <x:v>Thiếu staging live reconciliation</x:v>
+        <x:v>Cùng source-of-truth Dashboard; theo dõi khi API đổi contract</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -3179,13 +3179,13 @@
         <x:v>today/week/custom range, return order, site scope</x:v>
       </x:c>
       <x:c r="E6" s="86" t="str">
-        <x:v>Covered (mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F6" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="G6" s="68" t="str">
-        <x:v>Thiếu snapshot so với UI</x:v>
+        <x:v>Cùng source-of-truth Dashboard; theo dõi khi API đổi contract</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -3202,13 +3202,13 @@
         <x:v>top_n=1/10/100, pagination, zero rows</x:v>
       </x:c>
       <x:c r="E7" s="86" t="str">
-        <x:v>Covered (mock)</x:v>
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F7" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="G7" s="68" t="str">
-        <x:v>Thiếu UI reconciliation</x:v>
+        <x:v>Cùng source-of-truth Dashboard; theo dõi khi API đổi contract</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -3224,14 +3224,14 @@
       <x:c r="D8" s="67" t="str">
         <x:v>metric invalid, paging invalid, từng endpoint</x:v>
       </x:c>
-      <x:c r="E8" s="85" t="str">
-        <x:v>Partial</x:v>
+      <x:c r="E8" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F8" s="67" t="str">
-        <x:v>tests/test_dashboard_api.py</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="G8" s="68" t="str">
-        <x:v>Chỉ cover allow-list + một endpoint</x:v>
+        <x:v>Cùng source-of-truth Dashboard; theo dõi khi API đổi contract</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -3247,14 +3247,14 @@
       <x:c r="D9" s="67" t="str">
         <x:v>siteIds, customerIds, page/size, API 4xx</x:v>
       </x:c>
-      <x:c r="E9" s="84" t="str">
-        <x:v>Not covered</x:v>
+      <x:c r="E9" s="86" t="str">
+        <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F9" s="67" t="str">
-        <x:v>—</x:v>
+        <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
       <x:c r="G9" s="68" t="str">
-        <x:v>Ưu tiên thêm mock contract</x:v>
+        <x:v>Cùng source-of-truth Dashboard; theo dõi khi API đổi contract</x:v>
       </x:c>
     </x:row>
     <x:row r="10">

</xml_diff>

<commit_message>
Document dashboard API contracts in UAT checklist
</commit_message>
<xml_diff>
--- a/docs/Rocky_MCP_Technical_Checklist.xlsx
+++ b/docs/Rocky_MCP_Technical_Checklist.xlsx
@@ -2,11 +2,12 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R3affe759bb0d4255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R715d3223b7a3404e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R0eafba92967d403b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="R0b5934878fd0482f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R556821f016cf4e0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R8cd8f01e60da49b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R5b713f6232864323"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R017e4e62e9cd43b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Ra7544004061b4604"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R70c6fab8a4e44078"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="Rf348655c8c4c41e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3923,4 +3924,217 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="31" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="58" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+      <x:c r="B1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+      <x:c r="C1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+      <x:c r="D1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+      <x:c r="E1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="54"/>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="56" t="str">
+        <x:v>Tool MCP</x:v>
+      </x:c>
+      <x:c r="B3" s="56" t="str">
+        <x:v>REST endpoint read-only</x:v>
+      </x:c>
+      <x:c r="C3" s="56" t="str">
+        <x:v>Payload chính</x:v>
+      </x:c>
+      <x:c r="D3" s="56" t="str">
+        <x:v>Dữ liệu / công thức trả về</x:v>
+      </x:c>
+      <x:c r="E3" s="56" t="str">
+        <x:v>Quy tắc và giới hạn</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="61" t="str">
+        <x:v>get_dashboard_order_overview</x:v>
+      </x:c>
+      <x:c r="B4" s="62" t="str">
+        <x:v>POST /Admin/Dashboard/Order/Overview</x:v>
+      </x:c>
+      <x:c r="C4" s="62" t="str">
+        <x:v>periodType, startAt, endAt, siteIds, staffIds</x:v>
+      </x:c>
+      <x:c r="D4" s="62" t="str">
+        <x:v>4 KPI raw payload: số đơn, giá trị đơn, thực thu, còn phải thu</x:v>
+      </x:c>
+      <x:c r="E4" s="63" t="str">
+        <x:v>startAt/endAt = ngày VN (Asia/Ho_Chi_Minh) đổi epoch milliseconds; manager/BOD bị scope site.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="66" t="str">
+        <x:v>get_tinh_hinh_kinh_doanh</x:v>
+      </x:c>
+      <x:c r="B5" s="67" t="str">
+        <x:v>POST Order/Overview + POST Order/BySite; staff from POS</x:v>
+      </x:c>
+      <x:c r="C5" s="67" t="str">
+        <x:v>date range, siteIds</x:v>
+      </x:c>
+      <x:c r="D5" s="67" t="str">
+        <x:v>Tổng quan = overview Dashboard + theo chi nhánh Dashboard + ranking nhân viên POS</x:v>
+      </x:c>
+      <x:c r="E5" s="68" t="str">
+        <x:v>Tool tổng hợp; 4 KPI và site theo API Dashboard, staff không phải payload Dashboard.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="66" t="str">
+        <x:v>get_dashboard_order_by_site</x:v>
+      </x:c>
+      <x:c r="B6" s="67" t="str">
+        <x:v>POST /Admin/Dashboard/Order/BySite</x:v>
+      </x:c>
+      <x:c r="C6" s="67" t="str">
+        <x:v>periodType, startAt, endAt, siteIds</x:v>
+      </x:c>
+      <x:c r="D6" s="67" t="str">
+        <x:v>Raw doanh số theo chi nhánh như Dashboard</x:v>
+      </x:c>
+      <x:c r="E6" s="68" t="str">
+        <x:v>Không tự cộng/tính lại các card UI.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="66" t="str">
+        <x:v>get_dashboard_revenue</x:v>
+      </x:c>
+      <x:c r="B7" s="67" t="str">
+        <x:v>POST /Admin/Dashboard/Revenue</x:v>
+      </x:c>
+      <x:c r="C7" s="67" t="str">
+        <x:v>periodType, startAt, endAt, siteIds</x:v>
+      </x:c>
+      <x:c r="D7" s="67" t="str">
+        <x:v>summary.all.totalRevenue, hmkRevenue, otherRevenue, numOrder, numReturnOrder</x:v>
+      </x:c>
+      <x:c r="E7" s="68" t="str">
+        <x:v>Tổng doanh số Dashboard, không phải Thực thu/Còn phải thu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="66" t="str">
+        <x:v>get_revenue_by_source</x:v>
+      </x:c>
+      <x:c r="B8" s="67" t="str">
+        <x:v>POST /Admin/Dashboard/Revenue (alias)</x:v>
+      </x:c>
+      <x:c r="C8" s="67" t="str">
+        <x:v>periodType, startAt, endAt, siteIds</x:v>
+      </x:c>
+      <x:c r="D8" s="67" t="str">
+        <x:v>Forward cùng payload get_dashboard_revenue; phân tách HMK/Khác</x:v>
+      </x:c>
+      <x:c r="E8" s="68" t="str">
+        <x:v>Compatibility alias, nguồn chuẩn vẫn là Dashboard Revenue.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" s="66" t="str">
+        <x:v>get_dashboard_sales_by_customer</x:v>
+      </x:c>
+      <x:c r="B9" s="67" t="str">
+        <x:v>POST /Admin/Dashboard/Revenue/SalesByCustomer</x:v>
+      </x:c>
+      <x:c r="C9" s="67" t="str">
+        <x:v>fromDate, toDate, page=1, size=top_n</x:v>
+      </x:c>
+      <x:c r="D9" s="67" t="str">
+        <x:v>Tổng doanh số/số đơn/đơn trả = SUM các dòng Top N; số khách = meta.total</x:v>
+      </x:c>
+      <x:c r="E9" s="68" t="str">
+        <x:v>Không trộn tổng Top N với tổng toàn danh sách khách.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="66" t="str">
+        <x:v>get_dashboard_debt_overview</x:v>
+      </x:c>
+      <x:c r="B10" s="67" t="str">
+        <x:v>POST /Admin/DebtDashboard/RecoveryRate/Statistic + /Revenue/Statistic</x:v>
+      </x:c>
+      <x:c r="C10" s="67" t="str">
+        <x:v>startAt/endAt/customerIds; issueAt/paymentMethodIds</x:v>
+      </x:c>
+      <x:c r="D10" s="67" t="str">
+        <x:v>Số dư đầu kỳ, phát sinh, đã thu, tỷ lệ thu hồi và doanh thu nợ lấy trực tiếp response</x:v>
+      </x:c>
+      <x:c r="E10" s="68" t="str">
+        <x:v>Không thay bằng công thức PaymentOrder POS.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="66" t="str">
+        <x:v>get_dashboard_debt_customers</x:v>
+      </x:c>
+      <x:c r="B11" s="67" t="str">
+        <x:v>POST /Admin/DebtDashboard/CustomerDebt/GetPage</x:v>
+      </x:c>
+      <x:c r="C11" s="67" t="str">
+        <x:v>startAt, endAt, customerIds, page, size</x:v>
+      </x:c>
+      <x:c r="D11" s="67" t="str">
+        <x:v>Danh sách công nợ phân trang raw payload</x:v>
+      </x:c>
+      <x:c r="E11" s="68" t="str">
+        <x:v>page 1..10000; size 1..100.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="71" t="str">
+        <x:v>get_dashboard_metric</x:v>
+      </x:c>
+      <x:c r="B12" s="72" t="str">
+        <x:v>POST path theo DASHBOARD_READ_METRICS allow-list</x:v>
+      </x:c>
+      <x:c r="C12" s="72" t="str">
+        <x:v>Payload common hoặc revenue_list/staff/product; page, size</x:v>
+      </x:c>
+      <x:c r="D12" s="72" t="str">
+        <x:v>Forward raw payload endpoint theo metric; không có endpoint ghi</x:v>
+      </x:c>
+      <x:c r="E12" s="73" t="str">
+        <x:v>Allow-list hiện có 25 metric; code: dashboard_api.py:DASHBOARD_READ_METRICS.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:E1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
 </file>
</xml_diff>

<commit_message>
Add production smoke evidence and dashboard query contracts
</commit_message>
<xml_diff>
--- a/docs/Rocky_MCP_Technical_Checklist.xlsx
+++ b/docs/Rocky_MCP_Technical_Checklist.xlsx
@@ -2,12 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R8cd8f01e60da49b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R5b713f6232864323"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R017e4e62e9cd43b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Ra7544004061b4604"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R70c6fab8a4e44078"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="Rf348655c8c4c41e0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R53eeb17b077c4129"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R6235f492ab1c463f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R36365568b7564bf4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="R07b4de19695e4c4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R9873f6cb94714cfc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="R8778c590bfa64f06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Runtime smoke" sheetId="7" r:id="R7727ec895ce64558"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -226,7 +227,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="90">
+  <x:cellXfs count="92">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -436,6 +437,9 @@
     <x:xf numFmtId="0" fontId="0" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
@@ -455,6 +459,9 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="7" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
@@ -1074,7 +1081,7 @@
       <x:c r="H4" s="62" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I4" s="83" t="str">
+      <x:c r="I4" s="84" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J4" s="62" t="str">
@@ -1109,7 +1116,7 @@
       <x:c r="H5" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I5" s="84" t="str">
+      <x:c r="I5" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J5" s="67" t="str">
@@ -1144,7 +1151,7 @@
       <x:c r="H6" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I6" s="84" t="str">
+      <x:c r="I6" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J6" s="67" t="str">
@@ -1179,7 +1186,7 @@
       <x:c r="H7" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I7" s="84" t="str">
+      <x:c r="I7" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J7" s="67" t="str">
@@ -1214,7 +1221,7 @@
       <x:c r="H8" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I8" s="84" t="str">
+      <x:c r="I8" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J8" s="67" t="str">
@@ -1249,7 +1256,7 @@
       <x:c r="H9" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I9" s="84" t="str">
+      <x:c r="I9" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J9" s="67" t="str">
@@ -1284,7 +1291,7 @@
       <x:c r="H10" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I10" s="84" t="str">
+      <x:c r="I10" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J10" s="67" t="str">
@@ -1319,7 +1326,7 @@
       <x:c r="H11" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I11" s="84" t="str">
+      <x:c r="I11" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J11" s="67" t="str">
@@ -1354,7 +1361,7 @@
       <x:c r="H12" s="67" t="str">
         <x:v>tests/test_payment_types.py</x:v>
       </x:c>
-      <x:c r="I12" s="85" t="str">
+      <x:c r="I12" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J12" s="67" t="str">
@@ -1389,7 +1396,7 @@
       <x:c r="H13" s="67" t="str">
         <x:v>tests/test_payment_types.py</x:v>
       </x:c>
-      <x:c r="I13" s="85" t="str">
+      <x:c r="I13" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J13" s="67" t="str">
@@ -1424,7 +1431,7 @@
       <x:c r="H14" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I14" s="84" t="str">
+      <x:c r="I14" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J14" s="67" t="str">
@@ -1459,7 +1466,7 @@
       <x:c r="H15" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I15" s="84" t="str">
+      <x:c r="I15" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J15" s="67" t="str">
@@ -1494,7 +1501,7 @@
       <x:c r="H16" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I16" s="84" t="str">
+      <x:c r="I16" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J16" s="67" t="str">
@@ -1529,7 +1536,7 @@
       <x:c r="H17" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I17" s="84" t="str">
+      <x:c r="I17" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J17" s="67" t="str">
@@ -1564,7 +1571,7 @@
       <x:c r="H18" s="67" t="str">
         <x:v>tests/test_payment_types.py</x:v>
       </x:c>
-      <x:c r="I18" s="85" t="str">
+      <x:c r="I18" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J18" s="67" t="str">
@@ -1599,7 +1606,7 @@
       <x:c r="H19" s="67" t="str">
         <x:v>tests/test_payment_types.py</x:v>
       </x:c>
-      <x:c r="I19" s="85" t="str">
+      <x:c r="I19" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J19" s="67" t="str">
@@ -1634,7 +1641,7 @@
       <x:c r="H20" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I20" s="84" t="str">
+      <x:c r="I20" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J20" s="67" t="str">
@@ -1669,7 +1676,7 @@
       <x:c r="H21" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I21" s="84" t="str">
+      <x:c r="I21" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J21" s="67" t="str">
@@ -1704,7 +1711,7 @@
       <x:c r="H22" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I22" s="86" t="str">
+      <x:c r="I22" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J22" s="67" t="str">
@@ -1739,7 +1746,7 @@
       <x:c r="H23" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I23" s="84" t="str">
+      <x:c r="I23" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J23" s="67" t="str">
@@ -1774,7 +1781,7 @@
       <x:c r="H24" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I24" s="86" t="str">
+      <x:c r="I24" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J24" s="67" t="str">
@@ -1809,7 +1816,7 @@
       <x:c r="H25" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I25" s="86" t="str">
+      <x:c r="I25" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J25" s="67" t="str">
@@ -1844,7 +1851,7 @@
       <x:c r="H26" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I26" s="86" t="str">
+      <x:c r="I26" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J26" s="67" t="str">
@@ -1879,7 +1886,7 @@
       <x:c r="H27" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I27" s="86" t="str">
+      <x:c r="I27" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J27" s="67" t="str">
@@ -1914,7 +1921,7 @@
       <x:c r="H28" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I28" s="86" t="str">
+      <x:c r="I28" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J28" s="67" t="str">
@@ -1949,7 +1956,7 @@
       <x:c r="H29" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I29" s="86" t="str">
+      <x:c r="I29" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J29" s="67" t="str">
@@ -1984,7 +1991,7 @@
       <x:c r="H30" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I30" s="86" t="str">
+      <x:c r="I30" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J30" s="67" t="str">
@@ -2019,7 +2026,7 @@
       <x:c r="H31" s="67" t="str">
         <x:v>Dashboard API + tests/test_dashboard_api.py</x:v>
       </x:c>
-      <x:c r="I31" s="86" t="str">
+      <x:c r="I31" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="J31" s="67" t="str">
@@ -2054,7 +2061,7 @@
       <x:c r="H32" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I32" s="84" t="str">
+      <x:c r="I32" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J32" s="67" t="str">
@@ -2089,7 +2096,7 @@
       <x:c r="H33" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I33" s="84" t="str">
+      <x:c r="I33" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J33" s="67" t="str">
@@ -2124,7 +2131,7 @@
       <x:c r="H34" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I34" s="84" t="str">
+      <x:c r="I34" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J34" s="67" t="str">
@@ -2159,7 +2166,7 @@
       <x:c r="H35" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I35" s="84" t="str">
+      <x:c r="I35" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J35" s="67" t="str">
@@ -2194,7 +2201,7 @@
       <x:c r="H36" s="67" t="str">
         <x:v>tests/test_products_query.py</x:v>
       </x:c>
-      <x:c r="I36" s="86" t="str">
+      <x:c r="I36" s="87" t="str">
         <x:v>Covered (unit/mock)</x:v>
       </x:c>
       <x:c r="J36" s="67" t="str">
@@ -2229,7 +2236,7 @@
       <x:c r="H37" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I37" s="84" t="str">
+      <x:c r="I37" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J37" s="67" t="str">
@@ -2264,7 +2271,7 @@
       <x:c r="H38" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I38" s="84" t="str">
+      <x:c r="I38" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J38" s="67" t="str">
@@ -2299,7 +2306,7 @@
       <x:c r="H39" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I39" s="84" t="str">
+      <x:c r="I39" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J39" s="67" t="str">
@@ -2334,7 +2341,7 @@
       <x:c r="H40" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I40" s="84" t="str">
+      <x:c r="I40" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J40" s="67" t="str">
@@ -2369,7 +2376,7 @@
       <x:c r="H41" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I41" s="84" t="str">
+      <x:c r="I41" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J41" s="67" t="str">
@@ -2404,7 +2411,7 @@
       <x:c r="H42" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I42" s="84" t="str">
+      <x:c r="I42" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J42" s="67" t="str">
@@ -2439,7 +2446,7 @@
       <x:c r="H43" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I43" s="84" t="str">
+      <x:c r="I43" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J43" s="67" t="str">
@@ -2474,7 +2481,7 @@
       <x:c r="H44" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I44" s="84" t="str">
+      <x:c r="I44" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J44" s="67" t="str">
@@ -2509,7 +2516,7 @@
       <x:c r="H45" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I45" s="84" t="str">
+      <x:c r="I45" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J45" s="67" t="str">
@@ -2544,7 +2551,7 @@
       <x:c r="H46" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I46" s="84" t="str">
+      <x:c r="I46" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J46" s="67" t="str">
@@ -2579,7 +2586,7 @@
       <x:c r="H47" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I47" s="84" t="str">
+      <x:c r="I47" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J47" s="67" t="str">
@@ -2614,7 +2621,7 @@
       <x:c r="H48" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I48" s="84" t="str">
+      <x:c r="I48" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J48" s="67" t="str">
@@ -2649,7 +2656,7 @@
       <x:c r="H49" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I49" s="84" t="str">
+      <x:c r="I49" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J49" s="67" t="str">
@@ -2684,7 +2691,7 @@
       <x:c r="H50" s="67" t="str">
         <x:v>—</x:v>
       </x:c>
-      <x:c r="I50" s="84" t="str">
+      <x:c r="I50" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="J50" s="67" t="str">
@@ -2719,7 +2726,7 @@
       <x:c r="H51" s="67" t="str">
         <x:v>tests/test_disclaimers.py</x:v>
       </x:c>
-      <x:c r="I51" s="85" t="str">
+      <x:c r="I51" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J51" s="67" t="str">
@@ -2754,7 +2761,7 @@
       <x:c r="H52" s="67" t="str">
         <x:v>tests/test_disclaimers.py</x:v>
       </x:c>
-      <x:c r="I52" s="85" t="str">
+      <x:c r="I52" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J52" s="67" t="str">
@@ -2789,7 +2796,7 @@
       <x:c r="H53" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I53" s="85" t="str">
+      <x:c r="I53" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J53" s="67" t="str">
@@ -2824,7 +2831,7 @@
       <x:c r="H54" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I54" s="85" t="str">
+      <x:c r="I54" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J54" s="67" t="str">
@@ -2859,7 +2866,7 @@
       <x:c r="H55" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I55" s="85" t="str">
+      <x:c r="I55" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J55" s="67" t="str">
@@ -2894,7 +2901,7 @@
       <x:c r="H56" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I56" s="86" t="str">
+      <x:c r="I56" s="87" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="J56" s="67" t="str">
@@ -2929,7 +2936,7 @@
       <x:c r="H57" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I57" s="85" t="str">
+      <x:c r="I57" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="J57" s="67" t="str">
@@ -2964,7 +2971,7 @@
       <x:c r="H58" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I58" s="86" t="str">
+      <x:c r="I58" s="87" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="J58" s="67" t="str">
@@ -2999,7 +3006,7 @@
       <x:c r="H59" s="67" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I59" s="86" t="str">
+      <x:c r="I59" s="87" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="J59" s="67" t="str">
@@ -3034,7 +3041,7 @@
       <x:c r="H60" s="72" t="str">
         <x:v>tests/test_schema_retrieval.py</x:v>
       </x:c>
-      <x:c r="I60" s="87" t="str">
+      <x:c r="I60" s="88" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="J60" s="72" t="str">
@@ -3133,7 +3140,7 @@
       <x:c r="D4" s="62" t="str">
         <x:v>Unauthorized 401; BOD bị chặn tool ngoài allow-list; manager chỉ scope store</x:v>
       </x:c>
-      <x:c r="E4" s="88" t="str">
+      <x:c r="E4" s="89" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="F4" s="62" t="str">
@@ -3156,7 +3163,7 @@
       <x:c r="D5" s="67" t="str">
         <x:v>Ngày VN, site filter, staff filter, API lỗi</x:v>
       </x:c>
-      <x:c r="E5" s="86" t="str">
+      <x:c r="E5" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F5" s="67" t="str">
@@ -3179,7 +3186,7 @@
       <x:c r="D6" s="67" t="str">
         <x:v>today/week/custom range, return order, site scope</x:v>
       </x:c>
-      <x:c r="E6" s="86" t="str">
+      <x:c r="E6" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F6" s="67" t="str">
@@ -3202,7 +3209,7 @@
       <x:c r="D7" s="67" t="str">
         <x:v>top_n=1/10/100, pagination, zero rows</x:v>
       </x:c>
-      <x:c r="E7" s="86" t="str">
+      <x:c r="E7" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F7" s="67" t="str">
@@ -3225,7 +3232,7 @@
       <x:c r="D8" s="67" t="str">
         <x:v>metric invalid, paging invalid, từng endpoint</x:v>
       </x:c>
-      <x:c r="E8" s="86" t="str">
+      <x:c r="E8" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F8" s="67" t="str">
@@ -3248,7 +3255,7 @@
       <x:c r="D9" s="67" t="str">
         <x:v>siteIds, customerIds, page/size, API 4xx</x:v>
       </x:c>
-      <x:c r="E9" s="86" t="str">
+      <x:c r="E9" s="87" t="str">
         <x:v>Covered (API contract)</x:v>
       </x:c>
       <x:c r="F9" s="67" t="str">
@@ -3271,7 +3278,7 @@
       <x:c r="D10" s="67" t="str">
         <x:v>Allocate/Receive/invalid document type, range exclusive</x:v>
       </x:c>
-      <x:c r="E10" s="85" t="str">
+      <x:c r="E10" s="86" t="str">
         <x:v>Partial</x:v>
       </x:c>
       <x:c r="F10" s="67" t="str">
@@ -3294,7 +3301,7 @@
       <x:c r="D11" s="67" t="str">
         <x:v>date_field/state/code/customer, cancelled, paging</x:v>
       </x:c>
-      <x:c r="E11" s="84" t="str">
+      <x:c r="E11" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F11" s="67" t="str">
@@ -3317,7 +3324,7 @@
       <x:c r="D12" s="67" t="str">
         <x:v>zero denominator, return, ship, deleted/cancelled, store filter</x:v>
       </x:c>
-      <x:c r="E12" s="84" t="str">
+      <x:c r="E12" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F12" s="67" t="str">
@@ -3340,7 +3347,7 @@
       <x:c r="D13" s="67" t="str">
         <x:v>Top N, ties, missing product item</x:v>
       </x:c>
-      <x:c r="E13" s="86" t="str">
+      <x:c r="E13" s="87" t="str">
         <x:v>Covered (mock)</x:v>
       </x:c>
       <x:c r="F13" s="67" t="str">
@@ -3363,7 +3370,7 @@
       <x:c r="D14" s="67" t="str">
         <x:v>empty customer, negative balance, top limit</x:v>
       </x:c>
-      <x:c r="E14" s="84" t="str">
+      <x:c r="E14" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F14" s="67" t="str">
@@ -3386,7 +3393,7 @@
       <x:c r="D15" s="67" t="str">
         <x:v>WMS timeout, fallback cache, low stock, cancelled movement</x:v>
       </x:c>
-      <x:c r="E15" s="84" t="str">
+      <x:c r="E15" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F15" s="67" t="str">
@@ -3409,7 +3416,7 @@
       <x:c r="D16" s="67" t="str">
         <x:v>non-SELECT, multi statement, sensitive table, timeout</x:v>
       </x:c>
-      <x:c r="E16" s="84" t="str">
+      <x:c r="E16" s="85" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F16" s="67" t="str">
@@ -3432,7 +3439,7 @@
       <x:c r="D17" s="67" t="str">
         <x:v>unsafe table name, max results, file paging</x:v>
       </x:c>
-      <x:c r="E17" s="86" t="str">
+      <x:c r="E17" s="87" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="F17" s="67" t="str">
@@ -3455,7 +3462,7 @@
       <x:c r="D18" s="67" t="str">
         <x:v>Dashboard/WMS/legacy/raw/default output</x:v>
       </x:c>
-      <x:c r="E18" s="86" t="str">
+      <x:c r="E18" s="87" t="str">
         <x:v>Covered (unit)</x:v>
       </x:c>
       <x:c r="F18" s="67" t="str">
@@ -3478,7 +3485,7 @@
       <x:c r="D19" s="72" t="str">
         <x:v>no token, no mapping, failure, retry/idempotency</x:v>
       </x:c>
-      <x:c r="E19" s="89" t="str">
+      <x:c r="E19" s="90" t="str">
         <x:v>Not covered</x:v>
       </x:c>
       <x:c r="F19" s="72" t="str">
@@ -3935,6 +3942,7 @@
     <x:col min="3" max="3" width="52" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="72" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="58" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="68" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
@@ -3951,6 +3959,9 @@
         <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
       </x:c>
       <x:c r="E1" s="53" t="str">
+        <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
+      </x:c>
+      <x:c r="F1" s="53" t="str">
         <x:v>DASHBOARD API CONTRACT - ENDPOINT, PAYLOAD &amp; FORMULA</x:v>
       </x:c>
     </x:row>
@@ -3960,6 +3971,7 @@
       <x:c r="C2" s="54"/>
       <x:c r="D2" s="54"/>
       <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="56" t="str">
@@ -3977,6 +3989,9 @@
       <x:c r="E3" s="56" t="str">
         <x:v>Quy tắc và giới hạn</x:v>
       </x:c>
+      <x:c r="F3" s="56" t="str">
+        <x:v>Mẫu request / query formula</x:v>
+      </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="61" t="str">
@@ -3991,8 +4006,11 @@
       <x:c r="D4" s="62" t="str">
         <x:v>4 KPI raw payload: số đơn, giá trị đơn, thực thu, còn phải thu</x:v>
       </x:c>
-      <x:c r="E4" s="63" t="str">
+      <x:c r="E4" s="62" t="str">
         <x:v>startAt/endAt = ngày VN (Asia/Ho_Chi_Minh) đổi epoch milliseconds; manager/BOD bị scope site.</x:v>
+      </x:c>
+      <x:c r="F4" s="63" t="str">
+        <x:v>{periodType:1,startAt:&lt;epochVN&gt;,endAt:&lt;epochVN&gt;,siteIds:[...],staffIds:[...]}</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
@@ -4008,8 +4026,11 @@
       <x:c r="D5" s="67" t="str">
         <x:v>Tổng quan = overview Dashboard + theo chi nhánh Dashboard + ranking nhân viên POS</x:v>
       </x:c>
-      <x:c r="E5" s="68" t="str">
+      <x:c r="E5" s="67" t="str">
         <x:v>Tool tổng hợp; 4 KPI và site theo API Dashboard, staff không phải payload Dashboard.</x:v>
+      </x:c>
+      <x:c r="F5" s="68" t="str">
+        <x:v>overview(payload common) + bySite(payload common) + POS staff ranking</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -4025,8 +4046,11 @@
       <x:c r="D6" s="67" t="str">
         <x:v>Raw doanh số theo chi nhánh như Dashboard</x:v>
       </x:c>
-      <x:c r="E6" s="68" t="str">
+      <x:c r="E6" s="67" t="str">
         <x:v>Không tự cộng/tính lại các card UI.</x:v>
+      </x:c>
+      <x:c r="F6" s="68" t="str">
+        <x:v>{periodType:1,startAt:&lt;epochVN&gt;,endAt:&lt;epochVN&gt;,siteIds:[...]}</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -4042,8 +4066,11 @@
       <x:c r="D7" s="67" t="str">
         <x:v>summary.all.totalRevenue, hmkRevenue, otherRevenue, numOrder, numReturnOrder</x:v>
       </x:c>
-      <x:c r="E7" s="68" t="str">
+      <x:c r="E7" s="67" t="str">
         <x:v>Tổng doanh số Dashboard, không phải Thực thu/Còn phải thu.</x:v>
+      </x:c>
+      <x:c r="F7" s="68" t="str">
+        <x:v>{periodType:1,startAt:&lt;epochVN&gt;,endAt:&lt;epochVN&gt;,siteIds:[...]} → summary.all</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
@@ -4059,8 +4086,11 @@
       <x:c r="D8" s="67" t="str">
         <x:v>Forward cùng payload get_dashboard_revenue; phân tách HMK/Khác</x:v>
       </x:c>
-      <x:c r="E8" s="68" t="str">
+      <x:c r="E8" s="67" t="str">
         <x:v>Compatibility alias, nguồn chuẩn vẫn là Dashboard Revenue.</x:v>
+      </x:c>
+      <x:c r="F8" s="68" t="str">
+        <x:v>Cùng request Revenue → summary.all.{hmkRevenue,otherRevenue}</x:v>
       </x:c>
     </x:row>
     <x:row r="9">
@@ -4076,8 +4106,11 @@
       <x:c r="D9" s="67" t="str">
         <x:v>Tổng doanh số/số đơn/đơn trả = SUM các dòng Top N; số khách = meta.total</x:v>
       </x:c>
-      <x:c r="E9" s="68" t="str">
+      <x:c r="E9" s="67" t="str">
         <x:v>Không trộn tổng Top N với tổng toàn danh sách khách.</x:v>
+      </x:c>
+      <x:c r="F9" s="68" t="str">
+        <x:v>{fromDate:&lt;epochVN&gt;,toDate:&lt;epochVN&gt;,page:1,size:topN} → SUM(data[*])</x:v>
       </x:c>
     </x:row>
     <x:row r="10">
@@ -4093,8 +4126,11 @@
       <x:c r="D10" s="67" t="str">
         <x:v>Số dư đầu kỳ, phát sinh, đã thu, tỷ lệ thu hồi và doanh thu nợ lấy trực tiếp response</x:v>
       </x:c>
-      <x:c r="E10" s="68" t="str">
+      <x:c r="E10" s="67" t="str">
         <x:v>Không thay bằng công thức PaymentOrder POS.</x:v>
+      </x:c>
+      <x:c r="F10" s="68" t="str">
+        <x:v>recovery{startAt,endAt,customerIds} + revenue{issueAt:{from,to},customerIds,paymentMethodIds}</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
@@ -4110,8 +4146,11 @@
       <x:c r="D11" s="67" t="str">
         <x:v>Danh sách công nợ phân trang raw payload</x:v>
       </x:c>
-      <x:c r="E11" s="68" t="str">
+      <x:c r="E11" s="67" t="str">
         <x:v>page 1..10000; size 1..100.</x:v>
+      </x:c>
+      <x:c r="F11" s="68" t="str">
+        <x:v>{startAt:&lt;epochVN&gt;,endAt:&lt;epochVN&gt;,customerIds:[...],page,size}</x:v>
       </x:c>
     </x:row>
     <x:row r="12">
@@ -4127,13 +4166,164 @@
       <x:c r="D12" s="72" t="str">
         <x:v>Forward raw payload endpoint theo metric; không có endpoint ghi</x:v>
       </x:c>
-      <x:c r="E12" s="73" t="str">
+      <x:c r="E12" s="72" t="str">
         <x:v>Allow-list hiện có 25 metric; code: dashboard_api.py:DASHBOARD_READ_METRICS.</x:v>
+      </x:c>
+      <x:c r="F12" s="73" t="str">
+        <x:v>metric → allow-list path; common={periodType,startAt,endAt,siteIds,staffIds,...}</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
-    <x:mergeCell ref="A1:E1"/>
+    <x:mergeCell ref="A1:F1"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="43" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="70" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="16" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="62" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="28" customHeight="1">
+      <x:c r="A1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+      <x:c r="B1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+      <x:c r="C1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+      <x:c r="D1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+      <x:c r="E1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+      <x:c r="F1" s="53" t="str">
+        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" s="54"/>
+      <x:c r="B2" s="54"/>
+      <x:c r="C2" s="54"/>
+      <x:c r="D2" s="54"/>
+      <x:c r="E2" s="54"/>
+      <x:c r="F2" s="54"/>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" s="56" t="str">
+        <x:v>Thành phần</x:v>
+      </x:c>
+      <x:c r="B3" s="56" t="str">
+        <x:v>Probe</x:v>
+      </x:c>
+      <x:c r="C3" s="56" t="str">
+        <x:v>Evidence</x:v>
+      </x:c>
+      <x:c r="D3" s="56" t="str">
+        <x:v>Kết quả</x:v>
+      </x:c>
+      <x:c r="E3" s="56" t="str">
+        <x:v>Ngày test</x:v>
+      </x:c>
+      <x:c r="F3" s="56" t="str">
+        <x:v>Ghi chú</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" s="61" t="str">
+        <x:v>MCP endpoint + OAuth</x:v>
+      </x:c>
+      <x:c r="B4" s="62" t="str">
+        <x:v>https://rockyhmkmcp.share.zrok.io</x:v>
+      </x:c>
+      <x:c r="C4" s="62" t="str">
+        <x:v>Login 302; token 200; initialize 200</x:v>
+      </x:c>
+      <x:c r="D4" s="91" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="E4" s="62" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F4" s="63" t="str">
+        <x:v>Probe read-only qua OAuth; không ghi token hoặc thông tin bí mật.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="66" t="str">
+        <x:v>Dashboard API</x:v>
+      </x:c>
+      <x:c r="B5" s="67" t="str">
+        <x:v>get_dashboard_order_overview</x:v>
+      </x:c>
+      <x:c r="C5" s="67" t="str">
+        <x:v>HTTP 200; metric=dashboard_order_overview; source=rocky_dashboard_api</x:v>
+      </x:c>
+      <x:c r="D5" s="87" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="E5" s="67" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F5" s="68" t="str">
+        <x:v>Đọc KPI Dashboard qua REST API, không thay đổi dữ liệu.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="66" t="str">
+        <x:v>POS PostgreSQL</x:v>
+      </x:c>
+      <x:c r="B6" s="67" t="str">
+        <x:v>query_raw_pos_sql_tool: SELECT 1</x:v>
+      </x:c>
+      <x:c r="C6" s="67" t="str">
+        <x:v>HTTP 200; metric=raw_pos_sql</x:v>
+      </x:c>
+      <x:c r="D6" s="87" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="E6" s="67" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F6" s="68" t="str">
+        <x:v>Smoke SQL read-only, không đọc dữ liệu nghiệp vụ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="71" t="str">
+        <x:v>WMS PostgreSQL</x:v>
+      </x:c>
+      <x:c r="B7" s="72" t="str">
+        <x:v>check_wms_health</x:v>
+      </x:c>
+      <x:c r="C7" s="72" t="str">
+        <x:v>HTTP 200; status=ok; source=wms_live</x:v>
+      </x:c>
+      <x:c r="D7" s="88" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="E7" s="72" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F7" s="73" t="str">
+        <x:v>WMS live read-only health query.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:F1"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Clarify test coverage terminology in checklist
</commit_message>
<xml_diff>
--- a/docs/Rocky_MCP_Technical_Checklist.xlsx
+++ b/docs/Rocky_MCP_Technical_Checklist.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="R53eeb17b077c4129"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R6235f492ab1c463f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R36365568b7564bf4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="R07b4de19695e4c4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R9873f6cb94714cfc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="R8778c590bfa64f06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Runtime smoke" sheetId="7" r:id="R7727ec895ce64558"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="Rb4cbbf417b83499d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R6f33b0bcb0b7429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R79673e34210646dd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Rf3c759d738b3461f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R291077fc54a347c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="Rf725e8d554b94221"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Runtime smoke" sheetId="7" r:id="Rc538d0b6dcb94cdd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -905,7 +905,7 @@
     </x:row>
     <x:row r="12">
       <x:c r="A12" s="74" t="str">
-        <x:v>Kết luận hiện trạng: toàn bộ tool Dashboard API được nghiệm thu là ‘Covered (API contract)’ vì dùng cùng API/source-of-truth với giao diện Dashboard. Product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper có unit coverage. WMS, raw SQL safety, phần lớn vận hành POS/financial KPI và Telegram chưa có bộ test tự động đủ mạnh. ‘Covered (API contract)’ cần được rà lại khi Dashboard đổi API contract.</x:v>
+        <x:v>Quy ước quan trọng: ‘Not covered’ = chưa có test tự động hoặc evidence nghiệm thu cho tình huống đó; KHÔNG đồng nghĩa tool không chạy hoặc không kết nối được. Toàn bộ tool Dashboard API được nghiệm thu là ‘Covered (API contract)’ vì dùng cùng API/source-of-truth với giao diện Dashboard. Product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper có unit coverage. WMS, raw SQL safety, phần lớn vận hành POS/financial KPI và Telegram chưa có bộ test tự động đủ mạnh. ‘Covered (API contract)’ cần được rà lại khi Dashboard đổi API contract.</x:v>
       </x:c>
       <x:c r="B12" s="54"/>
       <x:c r="C12" s="54"/>
@@ -1047,7 +1047,7 @@
         <x:v>Evidence test</x:v>
       </x:c>
       <x:c r="I3" s="56" t="str">
-        <x:v>Coverage</x:v>
+        <x:v>Coverage test (không phải uptime)</x:v>
       </x:c>
       <x:c r="J3" s="56" t="str">
         <x:v>Gap / test cần bổ sung</x:v>
@@ -3118,7 +3118,7 @@
         <x:v>Các tình huống cần cover</x:v>
       </x:c>
       <x:c r="E3" s="56" t="str">
-        <x:v>Trạng thái hiện tại</x:v>
+        <x:v>Coverage test (không phải trạng thái chạy)</x:v>
       </x:c>
       <x:c r="F3" s="56" t="str">
         <x:v>Evidence</x:v>

</xml_diff>

<commit_message>
Update MCP runtime smoke checklist
</commit_message>
<xml_diff>
--- a/docs/Rocky_MCP_Technical_Checklist.xlsx
+++ b/docs/Rocky_MCP_Technical_Checklist.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="Rb4cbbf417b83499d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R6f33b0bcb0b7429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R79673e34210646dd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Rf3c759d738b3461f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R291077fc54a347c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="Rf725e8d554b94221"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Runtime smoke" sheetId="7" r:id="Rc538d0b6dcb94cdd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01 - Tổng quan" sheetId="1" r:id="Ra46873b0efcc4659"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="02 - Tool catalog" sheetId="2" r:id="R5874fbbccbf6455e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="03 - Test matrix" sheetId="3" r:id="R777c44f01c114803"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="04 - Data &amp; formula" sheetId="4" r:id="Rd2f88122b2c84daa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="05 - Gaps &amp; next steps" sheetId="5" r:id="R6c638cd62d594c18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="06 - Dashboard API" sheetId="6" r:id="R125fc6ebe5294944"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="07 - Runtime smoke" sheetId="7" r:id="R4b11895a15a04001"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -19,7 +19,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="8">
+  <x:fonts count="11">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -64,8 +64,26 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos Display"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF9C0006"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF006100"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF7F6000"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="8">
+  <x:fills count="11">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -100,6 +118,21 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFCE4D6"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFDE9D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2CC"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -227,7 +260,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="92">
+  <x:cellXfs count="100">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -463,6 +496,30 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="5" fillId="5" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -475,7 +532,7 @@
         <x:color rgb="FF9C0006"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE4D6"/>
         </x:patternFill>
       </x:fill>
@@ -486,7 +543,7 @@
         <x:color rgb="FF9C6500"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -903,17 +960,17 @@
       <x:c r="G11" s="54"/>
       <x:c r="H11" s="54"/>
     </x:row>
-    <x:row r="12">
+    <x:row r="12" ht="68" customHeight="1">
       <x:c r="A12" s="74" t="str">
-        <x:v>Quy ước quan trọng: ‘Not covered’ = chưa có test tự động hoặc evidence nghiệm thu cho tình huống đó; KHÔNG đồng nghĩa tool không chạy hoặc không kết nối được. Toàn bộ tool Dashboard API được nghiệm thu là ‘Covered (API contract)’ vì dùng cùng API/source-of-truth với giao diện Dashboard. Product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper có unit coverage. WMS, raw SQL safety, phần lớn vận hành POS/financial KPI và Telegram chưa có bộ test tự động đủ mạnh. ‘Covered (API contract)’ cần được rà lại khi Dashboard đổi API contract.</x:v>
-      </x:c>
-      <x:c r="B12" s="54"/>
-      <x:c r="C12" s="54"/>
-      <x:c r="D12" s="54"/>
-      <x:c r="E12" s="54"/>
-      <x:c r="F12" s="54"/>
-      <x:c r="G12" s="54"/>
-      <x:c r="H12" s="54"/>
+        <x:v>Quy ước quan trọng: ‘Not covered’ = chưa có test tự động hoặc evidence nghiệm thu cho tình huống đó; KHÔNG đồng nghĩa tool không chạy hoặc không kết nối được. Toàn bộ tool Dashboard API được nghiệm thu là ‘Covered (API contract)’ vì dùng cùng API/source-of-truth với giao diện Dashboard. Product ranking, schema retrieval, payment-type validation, local-auth migration và disclaimer helper có unit coverage. Runtime production 2026-08-18: lỗi BOM ở biến DASHBOARD_PG_DSN đã được vá; biến đã được nạp nhưng database Dashboard PG timeout mạng. Dashboard API, POS và WMS đều PASS qua probe read-only. 22 tool phụ thuộc Dashboard PG được đưa vào kế hoạch fallback trực tiếp theo nguồn, giữ nguyên tên tool và DSN MCP.</x:v>
+      </x:c>
+      <x:c r="B12" s="92"/>
+      <x:c r="C12" s="92"/>
+      <x:c r="D12" s="92"/>
+      <x:c r="E12" s="92"/>
+      <x:c r="F12" s="92"/>
+      <x:c r="G12" s="92"/>
+      <x:c r="H12" s="92"/>
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="54"/>
@@ -3921,6 +3978,23 @@
         <x:v>Sau UAT</x:v>
       </x:c>
     </x:row>
+    <x:row r="12" ht="58" customHeight="1">
+      <x:c r="A12" s="93" t="str">
+        <x:v>P0</x:v>
+      </x:c>
+      <x:c r="B12" s="93" t="str">
+        <x:v>Dashboard PG upstream connectivity</x:v>
+      </x:c>
+      <x:c r="C12" s="93" t="str">
+        <x:v>Sau khi vá BOM, Dashboard PG DSN đã được nạp nhưng connection timeout; 22 tool hiện phụ thuộc nguồn này không được coi là PASS runtime.</x:v>
+      </x:c>
+      <x:c r="D12" s="93" t="str">
+        <x:v>Giữ nguyên DSN và tool contract; ưu tiên fallback read-only theo Dashboard API/POS/WMS, test staging từng nhóm trước khi chuyển production. Raw Dashboard SQL và Telegram mapping chỉ khôi phục khi có nguồn tương đương hoặc DB kết nối lại.</x:v>
+      </x:c>
+      <x:c r="E12" s="93" t="str">
+        <x:v>Trước nghiệm thu lại 22 tool phụ thuộc Dashboard PG</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:E1"/>
@@ -4195,22 +4269,22 @@
   <x:sheetData>
     <x:row r="1" ht="28" customHeight="1">
       <x:c r="A1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
       <x:c r="B1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
       <x:c r="C1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
       <x:c r="D1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
       <x:c r="E1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
       <x:c r="F1" s="53" t="str">
-        <x:v>PRODUCTION READ-ONLY SMOKE - PASS RESULTS</x:v>
+        <x:v>PRODUCTION RUNTIME SMOKE - READ-ONLY RESULTS</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -4321,6 +4395,66 @@
         <x:v>WMS live read-only health query.</x:v>
       </x:c>
     </x:row>
+    <x:row r="8" ht="46" customHeight="1">
+      <x:c r="A8" s="93" t="str">
+        <x:v>Dashboard PostgreSQL runtime</x:v>
+      </x:c>
+      <x:c r="B8" s="93" t="str">
+        <x:v>query_raw_sql_tool: SELECT 1</x:v>
+      </x:c>
+      <x:c r="C8" s="93" t="str">
+        <x:v>BOM fix loaded DASHBOARD_PG_DSN; connection timeout after ~10s</x:v>
+      </x:c>
+      <x:c r="D8" s="95" t="str">
+        <x:v>BLOCKED - upstream connectivity</x:v>
+      </x:c>
+      <x:c r="E8" s="93" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F8" s="93" t="str">
+        <x:v>DSN không còn bị thiếu. Database Dashboard PG/đường mạng chưa phản hồi; không chạy truy vấn ghi hoặc restart thêm.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="46" customHeight="1">
+      <x:c r="A9" s="93" t="str">
+        <x:v>Direct read sources</x:v>
+      </x:c>
+      <x:c r="B9" s="93" t="str">
+        <x:v>Dashboard API + POS + WMS probes</x:v>
+      </x:c>
+      <x:c r="C9" s="93" t="str">
+        <x:v>Dashboard API HTTP 200; POS SELECT 1 HTTP 200; WMS health HTTP 200</x:v>
+      </x:c>
+      <x:c r="D9" s="97" t="str">
+        <x:v>PASS</x:v>
+      </x:c>
+      <x:c r="E9" s="93" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F9" s="93" t="str">
+        <x:v>Ba nguồn thay thế trực tiếp đang dùng read-only và là đích fallback cho tool nghiệp vụ.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="46" customHeight="1">
+      <x:c r="A10" s="93" t="str">
+        <x:v>Fallback migration</x:v>
+      </x:c>
+      <x:c r="B10" s="93" t="str">
+        <x:v>22 tool trước đây phụ thuộc Dashboard PG</x:v>
+      </x:c>
+      <x:c r="C10" s="93" t="str">
+        <x:v>Giữ nguyên tool name/role/DSN MCP; chuyển nội bộ theo Dashboard API, POS hoặc WMS; raw Dashboard SQL/Telegram mapping là ngoại lệ</x:v>
+      </x:c>
+      <x:c r="D10" s="99" t="str">
+        <x:v>IN PROGRESS</x:v>
+      </x:c>
+      <x:c r="E10" s="93" t="str">
+        <x:v>2026-08-18</x:v>
+      </x:c>
+      <x:c r="F10" s="93" t="str">
+        <x:v>Bắt buộc staging smoke và đối soát contract trước khi deploy production.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>

</xml_diff>